<commit_message>
3.1.32 Add virtualParams to common section of telegram for TypeReference.
</commit_message>
<xml_diff>
--- a/meta/program/BlancoRestGeneratorKtConstants.xlsx
+++ b/meta/program/BlancoRestGeneratorKtConstants.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10309"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10420"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/tueda/data/webstorm/blanco/blancoRestGeneratorKt/meta/program/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA4419BA-BE9C-7847-BD54-B1ABE2A2B604}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D395227-7A7B-E741-B73C-587A8E426819}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="500" windowWidth="33600" windowHeight="20500" tabRatio="640" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1219,7 +1219,7 @@
     <phoneticPr fontId="4"/>
   </si>
   <si>
-    <t>"3.1.31"</t>
+    <t>"3.1.32"</t>
     <phoneticPr fontId="4"/>
   </si>
 </sst>

</xml_diff>